<commit_message>
experiments results in pldi-23-rev
</commit_message>
<xml_diff>
--- a/docs/experiments.xlsx
+++ b/docs/experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sungkeunkim/git/DCCE/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F0B741-68A9-7F42-9FAB-2806FAEB8960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A9233E-F441-B740-98A3-978DA6FE5C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-8080" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{E6A628A0-BA48-FD4D-9B0A-CC4CBF8BF1CD}"/>
+    <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{E6A628A0-BA48-FD4D-9B0A-CC4CBF8BF1CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench status" sheetId="11" r:id="rId1"/>
@@ -863,15 +863,6 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -881,6 +872,15 @@
     <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1296,6 +1296,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1303,6 +1306,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1310,6 +1316,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1317,6 +1326,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1346,6 +1358,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1365,6 +1380,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1384,6 +1402,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1391,6 +1412,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1410,6 +1434,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1417,6 +1444,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1446,6 +1476,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1465,6 +1498,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1484,6 +1520,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1491,6 +1530,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000D-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1510,6 +1552,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000E-B466-0844-8284-BFB1EFEDB2A0}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:spPr>
@@ -2629,6 +2674,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2636,6 +2684,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2643,6 +2694,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2650,6 +2704,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2669,6 +2726,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2688,6 +2748,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2695,6 +2758,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2702,6 +2768,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2721,6 +2790,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2740,6 +2812,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2769,6 +2844,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2788,6 +2866,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -2795,6 +2876,9 @@
               <c:delete val="1"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-B74A-D240-9DAC-93CE07DA4624}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:spPr>
@@ -16338,7 +16422,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="61" t="s">
         <v>26</v>
       </c>
       <c r="B2" s="9" t="s">
@@ -16350,7 +16434,7 @@
       <c r="D2" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="E2" s="61" t="s">
         <v>67</v>
       </c>
       <c r="F2" s="15"/>
@@ -16359,7 +16443,7 @@
       <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>27</v>
       </c>
       <c r="B3" s="10" t="s">
@@ -16368,7 +16452,7 @@
       <c r="C3" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D3" s="62" t="s">
+      <c r="D3" s="59" t="s">
         <v>65</v>
       </c>
       <c r="E3" s="15"/>
@@ -16702,7 +16786,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A16" s="65" t="s">
+      <c r="A16" s="62" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="10" t="s">
@@ -16714,7 +16798,7 @@
       <c r="D16" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E16" s="64" t="s">
+      <c r="E16" s="61" t="s">
         <v>67</v>
       </c>
       <c r="F16" s="13"/>
@@ -16779,7 +16863,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="63" t="s">
+      <c r="A19" s="60" t="s">
         <v>38</v>
       </c>
       <c r="B19" s="10" t="s">
@@ -16788,7 +16872,7 @@
       <c r="C19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D19" s="62" t="s">
+      <c r="D19" s="59" t="s">
         <v>65</v>
       </c>
       <c r="E19" s="15"/>
@@ -16839,7 +16923,7 @@
       <c r="D21" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="64" t="s">
+      <c r="E21" s="61" t="s">
         <v>67</v>
       </c>
       <c r="F21" s="15"/>
@@ -16933,7 +17017,7 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A25" s="65" t="s">
+      <c r="A25" s="62" t="s">
         <v>9</v>
       </c>
       <c r="B25" s="10" t="s">
@@ -16945,7 +17029,7 @@
       <c r="D25" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E25" s="64" t="s">
+      <c r="E25" s="61" t="s">
         <v>67</v>
       </c>
       <c r="F25" s="15"/>
@@ -16954,7 +17038,7 @@
       <c r="I25" s="14"/>
     </row>
     <row r="26" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="60" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="10" t="s">
@@ -16963,7 +17047,7 @@
       <c r="C26" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="62" t="s">
+      <c r="D26" s="59" t="s">
         <v>65</v>
       </c>
       <c r="E26" s="15"/>
@@ -17357,7 +17441,7 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="18" x14ac:dyDescent="0.2">
-      <c r="A41" s="66" t="s">
+      <c r="A41" s="63" t="s">
         <v>18</v>
       </c>
       <c r="B41" s="12" t="s">
@@ -17369,7 +17453,7 @@
       <c r="D41" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E41" s="64" t="s">
+      <c r="E41" s="61" t="s">
         <v>67</v>
       </c>
       <c r="F41" s="15"/>
@@ -17860,17 +17944,17 @@
     </row>
     <row r="2" spans="2:17" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="8"/>
-      <c r="C2" s="59" t="s">
+      <c r="C2" s="70" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="60" t="s">
+      <c r="D2" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="61"/>
+      <c r="E2" s="69"/>
     </row>
     <row r="3" spans="2:17" ht="18" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="59"/>
+      <c r="C3" s="70"/>
       <c r="D3" s="6" t="s">
         <v>83</v>
       </c>
@@ -18335,7 +18419,7 @@
       <c r="B27" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="C27" s="67" t="s">
+      <c r="C27" s="64" t="s">
         <v>159</v>
       </c>
       <c r="D27" s="3">
@@ -20418,19 +20502,19 @@
       <c r="A6" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="B6" s="69">
+      <c r="B6" s="66">
         <v>38624</v>
       </c>
-      <c r="C6" s="69">
+      <c r="C6" s="66">
         <v>51535</v>
       </c>
-      <c r="D6" s="69">
+      <c r="D6" s="66">
         <v>114172</v>
       </c>
-      <c r="E6" s="69">
+      <c r="E6" s="66">
         <v>50575</v>
       </c>
-      <c r="F6" s="69">
+      <c r="F6" s="66">
         <v>55020</v>
       </c>
     </row>
@@ -20561,19 +20645,19 @@
       <c r="A13" s="58" t="s">
         <v>157</v>
       </c>
-      <c r="B13" s="69">
+      <c r="B13" s="66">
         <v>38444</v>
       </c>
-      <c r="C13" s="69">
+      <c r="C13" s="66">
         <v>51837</v>
       </c>
-      <c r="D13" s="69">
+      <c r="D13" s="66">
         <v>112813</v>
       </c>
-      <c r="E13" s="69">
+      <c r="E13" s="66">
         <v>51191</v>
       </c>
-      <c r="F13" s="69">
+      <c r="F13" s="66">
         <v>55299</v>
       </c>
     </row>
@@ -20817,23 +20901,23 @@
       <c r="A28" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="B28" s="68">
+      <c r="B28" s="65">
         <f t="shared" ref="B28:B35" si="4">B6/$B6</f>
         <v>1</v>
       </c>
-      <c r="C28" s="68">
+      <c r="C28" s="65">
         <f t="shared" ref="C28:F28" si="5">C6/$B6</f>
         <v>1.3342740265120132</v>
       </c>
-      <c r="D28" s="68">
+      <c r="D28" s="65">
         <f t="shared" si="5"/>
         <v>2.9559859154929575</v>
       </c>
-      <c r="E28" s="68">
+      <c r="E28" s="65">
         <f t="shared" si="5"/>
         <v>1.309419014084507</v>
       </c>
-      <c r="F28" s="68">
+      <c r="F28" s="65">
         <f t="shared" si="5"/>
         <v>1.4245028997514499</v>
       </c>
@@ -21013,23 +21097,23 @@
       <c r="A35" s="58" t="s">
         <v>157</v>
       </c>
-      <c r="B35" s="68">
+      <c r="B35" s="65">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="C35" s="68">
+      <c r="C35" s="65">
         <f t="shared" ref="C35:F35" si="12">C13/$B13</f>
         <v>1.3483768598480907</v>
       </c>
-      <c r="D35" s="68">
+      <c r="D35" s="65">
         <f t="shared" si="12"/>
         <v>2.9344761211112269</v>
       </c>
-      <c r="E35" s="68">
+      <c r="E35" s="65">
         <f t="shared" si="12"/>
         <v>1.3315731973780043</v>
       </c>
-      <c r="F35" s="68">
+      <c r="F35" s="65">
         <f t="shared" si="12"/>
         <v>1.4384299240453646</v>
       </c>
@@ -21284,15 +21368,15 @@
         <v>0.45703125</v>
       </c>
       <c r="H48" s="20">
-        <f>(D48-$B48)/1024</f>
+        <f t="shared" ref="H48:I50" si="20">(D48-$B48)/1024</f>
         <v>1.21875</v>
       </c>
       <c r="I48" s="20">
-        <f>(E48-$B48)/1024</f>
+        <f t="shared" si="20"/>
         <v>0.515625</v>
       </c>
       <c r="J48" s="20">
-        <f t="shared" ref="J48:J61" si="20">(F48-$B48)/1024</f>
+        <f t="shared" ref="J48:J61" si="21">(F48-$B48)/1024</f>
         <v>0.4609375</v>
       </c>
       <c r="K48" s="25"/>
@@ -21321,15 +21405,15 @@
         <v>1.51953125</v>
       </c>
       <c r="H49" s="20">
-        <f>(D49-$B49)/1024</f>
+        <f t="shared" si="20"/>
         <v>3.70703125</v>
       </c>
       <c r="I49" s="20">
-        <f>(E49-$B49)/1024</f>
+        <f t="shared" si="20"/>
         <v>1.15625</v>
       </c>
       <c r="J49" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1.1796875</v>
       </c>
       <c r="K49" s="25"/>
@@ -21358,15 +21442,15 @@
         <v>1.9609375</v>
       </c>
       <c r="H50" s="20">
-        <f>(D50-$B50)/1024</f>
+        <f t="shared" si="20"/>
         <v>2.04296875</v>
       </c>
       <c r="I50" s="20">
-        <f>(E50-$B50)/1024</f>
+        <f t="shared" si="20"/>
         <v>1.58984375</v>
       </c>
       <c r="J50" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1.6171875</v>
       </c>
       <c r="K50" s="25"/>
@@ -21375,35 +21459,35 @@
       <c r="A51" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="B51" s="69">
+      <c r="B51" s="66">
         <v>247416</v>
       </c>
-      <c r="C51" s="69">
+      <c r="C51" s="66">
         <v>249712</v>
       </c>
-      <c r="D51" s="69">
+      <c r="D51" s="66">
         <v>249712</v>
       </c>
-      <c r="E51" s="69">
+      <c r="E51" s="66">
         <v>249136</v>
       </c>
-      <c r="F51" s="69">
+      <c r="F51" s="66">
         <v>249200</v>
       </c>
-      <c r="G51" s="68">
-        <f t="shared" ref="G51:G58" si="21">(C51-$B51)/1024</f>
+      <c r="G51" s="65">
+        <f t="shared" ref="G51:G58" si="22">(C51-$B51)/1024</f>
         <v>2.2421875</v>
       </c>
-      <c r="H51" s="68">
-        <f t="shared" ref="H51:H58" si="22">(D51-$B51)/1024</f>
+      <c r="H51" s="65">
+        <f t="shared" ref="H51:H58" si="23">(D51-$B51)/1024</f>
         <v>2.2421875</v>
       </c>
-      <c r="I51" s="68">
-        <f t="shared" ref="I51:I58" si="23">(E51-$B51)/1024</f>
+      <c r="I51" s="65">
+        <f t="shared" ref="I51:I58" si="24">(E51-$B51)/1024</f>
         <v>1.6796875</v>
       </c>
-      <c r="J51" s="68">
-        <f t="shared" ref="J51:J58" si="24">(F51-$B51)/1024</f>
+      <c r="J51" s="65">
+        <f t="shared" ref="J51:J58" si="25">(F51-$B51)/1024</f>
         <v>1.7421875</v>
       </c>
       <c r="K51" s="25"/>
@@ -21428,19 +21512,19 @@
         <v>494656</v>
       </c>
       <c r="G52" s="20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>4.4453125</v>
       </c>
       <c r="H52" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>13.62890625</v>
       </c>
       <c r="I52" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>3.67578125</v>
       </c>
       <c r="J52" s="20">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>3.921875</v>
       </c>
       <c r="K52" s="25"/>
@@ -21465,19 +21549,19 @@
         <v>162660</v>
       </c>
       <c r="G53" s="20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.6171875</v>
       </c>
       <c r="H53" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>7.55859375</v>
       </c>
       <c r="I53" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>2.44140625</v>
       </c>
       <c r="J53" s="20">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>2.64453125</v>
       </c>
       <c r="K53" s="25"/>
@@ -21502,19 +21586,19 @@
         <v>28296</v>
       </c>
       <c r="G54" s="20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0.703125</v>
       </c>
       <c r="H54" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>1.9453125</v>
       </c>
       <c r="I54" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0.6484375</v>
       </c>
       <c r="J54" s="20">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.63671875</v>
       </c>
       <c r="K54" s="25"/>
@@ -21539,19 +21623,19 @@
         <v>745524</v>
       </c>
       <c r="G55" s="20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.40625</v>
       </c>
       <c r="H55" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>2.91796875</v>
       </c>
       <c r="I55" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>2.32421875</v>
       </c>
       <c r="J55" s="20">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>2.4609375</v>
       </c>
       <c r="K55" s="25"/>
@@ -21576,19 +21660,19 @@
         <v>4058300</v>
       </c>
       <c r="G56" s="20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>1.66796875</v>
       </c>
       <c r="H56" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>1.75390625</v>
       </c>
       <c r="I56" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1.53515625</v>
       </c>
       <c r="J56" s="20">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>1.609375</v>
       </c>
       <c r="K56" s="25"/>
@@ -21613,19 +21697,19 @@
         <v>3303576</v>
       </c>
       <c r="G57" s="20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>1.45703125</v>
       </c>
       <c r="H57" s="20">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>1.65625</v>
       </c>
       <c r="I57" s="20">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>1.39453125</v>
       </c>
       <c r="J57" s="20">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>1.3046875</v>
       </c>
       <c r="K57" s="25"/>
@@ -21634,35 +21718,35 @@
       <c r="A58" s="58" t="s">
         <v>157</v>
       </c>
-      <c r="B58" s="69">
+      <c r="B58" s="66">
         <v>247668</v>
       </c>
-      <c r="C58" s="69">
+      <c r="C58" s="66">
         <v>249648</v>
       </c>
-      <c r="D58" s="69">
+      <c r="D58" s="66">
         <v>249776</v>
       </c>
-      <c r="E58" s="69">
+      <c r="E58" s="66">
         <v>249136</v>
       </c>
-      <c r="F58" s="69">
+      <c r="F58" s="66">
         <v>249200</v>
       </c>
-      <c r="G58" s="68">
-        <f t="shared" si="21"/>
+      <c r="G58" s="65">
+        <f t="shared" si="22"/>
         <v>1.93359375</v>
       </c>
-      <c r="H58" s="68">
-        <f t="shared" si="22"/>
+      <c r="H58" s="65">
+        <f t="shared" si="23"/>
         <v>2.05859375</v>
       </c>
-      <c r="I58" s="68">
-        <f t="shared" si="23"/>
+      <c r="I58" s="65">
+        <f t="shared" si="24"/>
         <v>1.43359375</v>
       </c>
-      <c r="J58" s="68">
-        <f t="shared" si="24"/>
+      <c r="J58" s="65">
+        <f t="shared" si="25"/>
         <v>1.49609375</v>
       </c>
       <c r="K58" s="25"/>
@@ -21691,15 +21775,15 @@
         <v>3.9921875</v>
       </c>
       <c r="H59" s="20">
-        <f>(D59-$B59)/1024</f>
+        <f t="shared" ref="H59:I61" si="26">(D59-$B59)/1024</f>
         <v>13.20703125</v>
       </c>
       <c r="I59" s="20">
-        <f>(E59-$B59)/1024</f>
+        <f t="shared" si="26"/>
         <v>3.359375</v>
       </c>
       <c r="J59" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>3.56640625</v>
       </c>
       <c r="K59" s="25"/>
@@ -21728,15 +21812,15 @@
         <v>2.40234375</v>
       </c>
       <c r="H60" s="20">
-        <f>(D60-$B60)/1024</f>
+        <f t="shared" si="26"/>
         <v>7.21875</v>
       </c>
       <c r="I60" s="20">
-        <f>(E60-$B60)/1024</f>
+        <f t="shared" si="26"/>
         <v>2.34765625</v>
       </c>
       <c r="J60" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>2.3671875</v>
       </c>
       <c r="K60" s="25"/>
@@ -21765,15 +21849,15 @@
         <v>0.37109375</v>
       </c>
       <c r="H61" s="20">
-        <f>(D61-$B61)/1024</f>
+        <f t="shared" si="26"/>
         <v>0.5390625</v>
       </c>
       <c r="I61" s="20">
-        <f>(E61-$B61)/1024</f>
+        <f t="shared" si="26"/>
         <v>0.19140625</v>
       </c>
       <c r="J61" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0.2421875</v>
       </c>
       <c r="K61" s="25"/>
@@ -22117,19 +22201,19 @@
       <c r="A12" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B12" s="69">
+      <c r="B12" s="66">
         <v>5884</v>
       </c>
-      <c r="C12" s="69">
+      <c r="C12" s="66">
         <v>6102</v>
       </c>
-      <c r="D12" s="69">
+      <c r="D12" s="66">
         <v>15728</v>
       </c>
-      <c r="E12" s="69">
+      <c r="E12" s="66">
         <v>6319</v>
       </c>
-      <c r="F12" s="69">
+      <c r="F12" s="66">
         <v>6940</v>
       </c>
     </row>
@@ -22201,23 +22285,23 @@
         <v>91</v>
       </c>
       <c r="B18" s="20">
-        <f>B2/$B2</f>
+        <f t="shared" ref="B18:B30" si="0">B2/$B2</f>
         <v>1</v>
       </c>
       <c r="C18" s="20">
-        <f t="shared" ref="C18:F18" si="0">C2/$B2</f>
+        <f t="shared" ref="C18:F18" si="1">C2/$B2</f>
         <v>2.1923076923076925</v>
       </c>
       <c r="D18" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>15.76923076923077</v>
       </c>
       <c r="E18" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.7307692307692308</v>
       </c>
       <c r="F18" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.8461538461538463</v>
       </c>
       <c r="G18" s="21"/>
@@ -22230,23 +22314,23 @@
         <v>92</v>
       </c>
       <c r="B19" s="20">
-        <f>B3/$B3</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C19" s="20">
-        <f t="shared" ref="C19:F19" si="1">C3/$B3</f>
+        <f t="shared" ref="C19:F19" si="2">C3/$B3</f>
         <v>1.0454545454545454</v>
       </c>
       <c r="D19" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.6363636363636362</v>
       </c>
       <c r="E19" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.0909090909090908</v>
       </c>
       <c r="F19" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.1363636363636365</v>
       </c>
       <c r="G19" s="21"/>
@@ -22259,23 +22343,23 @@
         <v>93</v>
       </c>
       <c r="B20" s="20">
-        <f>B4/$B4</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C20" s="20">
-        <f t="shared" ref="C20:F20" si="2">C4/$B4</f>
+        <f t="shared" ref="C20:F20" si="3">C4/$B4</f>
         <v>1.0241137304300882</v>
       </c>
       <c r="D20" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.5805290624437647</v>
       </c>
       <c r="E20" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1693359726471118</v>
       </c>
       <c r="F20" s="20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1182292603922981</v>
       </c>
       <c r="G20" s="21"/>
@@ -22288,23 +22372,23 @@
         <v>94</v>
       </c>
       <c r="B21" s="20">
-        <f>B5/$B5</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C21" s="20">
-        <f t="shared" ref="C21:F21" si="3">C5/$B5</f>
+        <f t="shared" ref="C21:F21" si="4">C5/$B5</f>
         <v>0.93181818181818177</v>
       </c>
       <c r="D21" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.7045454545454546</v>
       </c>
       <c r="E21" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.95454545454545459</v>
       </c>
       <c r="F21" s="20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.97727272727272729</v>
       </c>
       <c r="G21" s="21"/>
@@ -22317,23 +22401,23 @@
         <v>95</v>
       </c>
       <c r="B22" s="20">
-        <f>B6/$B6</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C22" s="20">
-        <f t="shared" ref="C22:F22" si="4">C6/$B6</f>
+        <f t="shared" ref="C22:F22" si="5">C6/$B6</f>
         <v>1.7817142857142858</v>
       </c>
       <c r="D22" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>11.063619047619047</v>
       </c>
       <c r="E22" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.8213333333333332</v>
       </c>
       <c r="F22" s="20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.7344761904761905</v>
       </c>
       <c r="G22" s="21"/>
@@ -22346,23 +22430,23 @@
         <v>96</v>
       </c>
       <c r="B23" s="20">
-        <f>B7/$B7</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C23" s="20">
-        <f t="shared" ref="C23:F23" si="5">C7/$B7</f>
+        <f t="shared" ref="C23:F23" si="6">C7/$B7</f>
         <v>1.5210866752910737</v>
       </c>
       <c r="D23" s="20">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>7.9055627425614485</v>
       </c>
       <c r="E23" s="20">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1.4271668822768435</v>
       </c>
       <c r="F23" s="20">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1.5060802069857697</v>
       </c>
       <c r="G23" s="21"/>
@@ -22375,23 +22459,23 @@
         <v>97</v>
       </c>
       <c r="B24" s="20">
-        <f>B8/$B8</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C24" s="20">
-        <f t="shared" ref="C24:F24" si="6">C8/$B8</f>
+        <f t="shared" ref="C24:F24" si="7">C8/$B8</f>
         <v>1.0066334991708126</v>
       </c>
       <c r="D24" s="20">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1.0182421227197347</v>
       </c>
       <c r="E24" s="20">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1.0071862907683804</v>
       </c>
       <c r="F24" s="20">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1.007739082365948</v>
       </c>
       <c r="G24" s="21"/>
@@ -22404,23 +22488,23 @@
         <v>98</v>
       </c>
       <c r="B25" s="20">
-        <f>B9/$B9</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C25" s="20">
-        <f t="shared" ref="C25:F25" si="7">C9/$B9</f>
+        <f t="shared" ref="C25:F25" si="8">C9/$B9</f>
         <v>0.97901168969181718</v>
       </c>
       <c r="D25" s="20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.98618490967056327</v>
       </c>
       <c r="E25" s="20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.98591923485653565</v>
       </c>
       <c r="F25" s="20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.0092986184909671</v>
       </c>
       <c r="G25" s="21"/>
@@ -22433,23 +22517,23 @@
         <v>99</v>
       </c>
       <c r="B26" s="20">
-        <f>B10/$B10</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C26" s="20">
-        <f t="shared" ref="C26:F26" si="8">C10/$B10</f>
+        <f t="shared" ref="C26:F26" si="9">C10/$B10</f>
         <v>2.6774193548387095</v>
       </c>
       <c r="D26" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>28.838709677419356</v>
       </c>
       <c r="E26" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>3.161290322580645</v>
       </c>
       <c r="F26" s="20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>3.4193548387096775</v>
       </c>
       <c r="G26" s="21"/>
@@ -22462,23 +22546,23 @@
         <v>100</v>
       </c>
       <c r="B27" s="20">
-        <f>B11/$B11</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C27" s="20">
-        <f t="shared" ref="C27:F27" si="9">C11/$B11</f>
+        <f t="shared" ref="C27:F27" si="10">C11/$B11</f>
         <v>1.3530031612223392</v>
       </c>
       <c r="D27" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>8.1707060063224439</v>
       </c>
       <c r="E27" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1.3582718651211803</v>
       </c>
       <c r="F27" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1.3909378292939938</v>
       </c>
       <c r="G27" s="21"/>
@@ -22490,24 +22574,24 @@
       <c r="A28" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B28" s="68">
-        <f>B12/$B12</f>
+      <c r="B28" s="65">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="C28" s="68">
-        <f t="shared" ref="C28:F28" si="10">C12/$B12</f>
+      <c r="C28" s="65">
+        <f t="shared" ref="C28:F28" si="11">C12/$B12</f>
         <v>1.0370496261046906</v>
       </c>
-      <c r="D28" s="68">
-        <f t="shared" si="10"/>
+      <c r="D28" s="65">
+        <f t="shared" si="11"/>
         <v>2.6730115567641062</v>
       </c>
-      <c r="E28" s="68">
-        <f t="shared" si="10"/>
+      <c r="E28" s="65">
+        <f t="shared" si="11"/>
         <v>1.073929299796057</v>
       </c>
-      <c r="F28" s="68">
-        <f t="shared" si="10"/>
+      <c r="F28" s="65">
+        <f t="shared" si="11"/>
         <v>1.1794697484704282</v>
       </c>
       <c r="G28" s="21"/>
@@ -22520,23 +22604,23 @@
         <v>101</v>
       </c>
       <c r="B29" s="20">
-        <f>B13/$B13</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C29" s="20">
-        <f t="shared" ref="C29:F29" si="11">C13/$B13</f>
+        <f t="shared" ref="C29:F29" si="12">C13/$B13</f>
         <v>1.3771186440677967</v>
       </c>
       <c r="D29" s="20">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.8919491525423728</v>
       </c>
       <c r="E29" s="20">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.4682203389830508</v>
       </c>
       <c r="F29" s="20">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.6271186440677967</v>
       </c>
       <c r="G29" s="21"/>
@@ -22549,23 +22633,23 @@
         <v>102</v>
       </c>
       <c r="B30" s="20">
-        <f>B14/$B14</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C30" s="20">
-        <f t="shared" ref="C30:F30" si="12">C14/$B14</f>
+        <f t="shared" ref="C30:F30" si="13">C14/$B14</f>
         <v>1.5</v>
       </c>
       <c r="D30" s="20">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6.2777777777777777</v>
       </c>
       <c r="E30" s="20">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1.537037037037037</v>
       </c>
       <c r="F30" s="20">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1.6851851851851851</v>
       </c>
       <c r="G30" s="21"/>
@@ -22582,7 +22666,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="20">
-        <f t="shared" ref="C31" si="13">GEOMEAN(C18:C30)</f>
+        <f t="shared" ref="C31" si="14">GEOMEAN(C18:C30)</f>
         <v>1.3409621318138527</v>
       </c>
       <c r="D31" s="20">
@@ -22690,11 +22774,11 @@
         <v>1.8203125</v>
       </c>
       <c r="H40" s="26">
-        <f>(E40-$B40)/1024</f>
+        <f t="shared" ref="H40:H52" si="15">(E40-$B40)/1024</f>
         <v>1.4921875</v>
       </c>
       <c r="I40" s="26">
-        <f>(D40-$B40)/1024</f>
+        <f t="shared" ref="I40:I52" si="16">(D40-$B40)/1024</f>
         <v>1.75390625</v>
       </c>
       <c r="J40" s="26">
@@ -22702,7 +22786,7 @@
         <v>1.48828125</v>
       </c>
       <c r="K40" s="25">
-        <f t="shared" ref="K40:K52" si="14">I40-J40</f>
+        <f t="shared" ref="K40:K52" si="17">I40-J40</f>
         <v>0.265625</v>
       </c>
     </row>
@@ -22726,23 +22810,23 @@
         <v>43944</v>
       </c>
       <c r="G41" s="26">
-        <f t="shared" ref="G41:G52" si="15">(C41-$B41)/1024</f>
+        <f t="shared" ref="G41:G52" si="18">(C41-$B41)/1024</f>
         <v>2.48046875</v>
       </c>
       <c r="H41" s="26">
-        <f>(E41-$B41)/1024</f>
+        <f t="shared" si="15"/>
         <v>2.4140625</v>
       </c>
       <c r="I41" s="26">
-        <f>(D41-$B41)/1024</f>
+        <f t="shared" si="16"/>
         <v>2.2421875</v>
       </c>
       <c r="J41" s="26">
-        <f t="shared" ref="J41:J52" si="16">(F41-$B41)/1024</f>
+        <f t="shared" ref="J41:J52" si="19">(F41-$B41)/1024</f>
         <v>2.3515625</v>
       </c>
       <c r="K41" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>-0.109375</v>
       </c>
     </row>
@@ -22766,23 +22850,23 @@
         <v>12588864</v>
       </c>
       <c r="G42" s="26">
+        <f t="shared" si="18"/>
+        <v>1.95703125</v>
+      </c>
+      <c r="H42" s="26">
         <f t="shared" si="15"/>
-        <v>1.95703125</v>
-      </c>
-      <c r="H42" s="26">
-        <f>(E42-$B42)/1024</f>
         <v>1.8828125</v>
       </c>
       <c r="I42" s="26">
-        <f>(D42-$B42)/1024</f>
+        <f t="shared" si="16"/>
         <v>1.9765625</v>
       </c>
       <c r="J42" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.6796875</v>
       </c>
       <c r="K42" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.296875</v>
       </c>
     </row>
@@ -22806,23 +22890,23 @@
         <v>27744</v>
       </c>
       <c r="G43" s="26">
+        <f t="shared" si="18"/>
+        <v>1.703125</v>
+      </c>
+      <c r="H43" s="26">
         <f t="shared" si="15"/>
-        <v>1.703125</v>
-      </c>
-      <c r="H43" s="26">
-        <f>(E43-$B43)/1024</f>
         <v>1.4140625</v>
       </c>
       <c r="I43" s="26">
-        <f>(D43-$B43)/1024</f>
+        <f t="shared" si="16"/>
         <v>1.67578125</v>
       </c>
       <c r="J43" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.50390625</v>
       </c>
       <c r="K43" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.171875</v>
       </c>
     </row>
@@ -22846,23 +22930,23 @@
         <v>135804</v>
       </c>
       <c r="G44" s="26">
+        <f t="shared" si="18"/>
+        <v>1.91015625</v>
+      </c>
+      <c r="H44" s="26">
         <f t="shared" si="15"/>
-        <v>1.91015625</v>
-      </c>
-      <c r="H44" s="26">
-        <f>(E44-$B44)/1024</f>
         <v>1.76953125</v>
       </c>
       <c r="I44" s="26">
-        <f>(D44-$B44)/1024</f>
+        <f t="shared" si="16"/>
         <v>1.890625</v>
       </c>
       <c r="J44" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.796875</v>
       </c>
       <c r="K44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>9.375E-2</v>
       </c>
     </row>
@@ -22886,23 +22970,23 @@
         <v>135344</v>
       </c>
       <c r="G45" s="26">
+        <f t="shared" si="18"/>
+        <v>1.91796875</v>
+      </c>
+      <c r="H45" s="26">
         <f t="shared" si="15"/>
-        <v>1.91796875</v>
-      </c>
-      <c r="H45" s="26">
-        <f>(E45-$B45)/1024</f>
         <v>1.7734375</v>
       </c>
       <c r="I45" s="26">
-        <f>(D45-$B45)/1024</f>
+        <f t="shared" si="16"/>
         <v>2.05078125</v>
       </c>
       <c r="J45" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.859375</v>
       </c>
       <c r="K45" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.19140625</v>
       </c>
     </row>
@@ -22926,23 +23010,23 @@
         <v>3631688</v>
       </c>
       <c r="G46" s="26">
+        <f t="shared" si="18"/>
+        <v>1.9921875</v>
+      </c>
+      <c r="H46" s="26">
         <f t="shared" si="15"/>
-        <v>1.9921875</v>
-      </c>
-      <c r="H46" s="26">
-        <f>(E46-$B46)/1024</f>
         <v>2.00390625</v>
       </c>
       <c r="I46" s="26">
-        <f>(D46-$B46)/1024</f>
+        <f t="shared" si="16"/>
         <v>2.07421875</v>
       </c>
       <c r="J46" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.90625</v>
       </c>
       <c r="K46" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.16796875</v>
       </c>
     </row>
@@ -22966,23 +23050,23 @@
         <v>4094376</v>
       </c>
       <c r="G47" s="26">
+        <f t="shared" si="18"/>
+        <v>1.890625</v>
+      </c>
+      <c r="H47" s="26">
         <f t="shared" si="15"/>
-        <v>1.890625</v>
-      </c>
-      <c r="H47" s="26">
-        <f>(E47-$B47)/1024</f>
         <v>1.8828125</v>
       </c>
       <c r="I47" s="26">
-        <f>(D47-$B47)/1024</f>
+        <f t="shared" si="16"/>
         <v>1.94140625</v>
       </c>
       <c r="J47" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.66796875</v>
       </c>
       <c r="K47" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.2734375</v>
       </c>
     </row>
@@ -23006,23 +23090,23 @@
         <v>220900</v>
       </c>
       <c r="G48" s="26">
+        <f t="shared" si="18"/>
+        <v>1.80078125</v>
+      </c>
+      <c r="H48" s="26">
         <f t="shared" si="15"/>
-        <v>1.80078125</v>
-      </c>
-      <c r="H48" s="26">
-        <f>(E48-$B48)/1024</f>
         <v>1.5234375</v>
       </c>
       <c r="I48" s="26">
-        <f>(D48-$B48)/1024</f>
+        <f t="shared" si="16"/>
         <v>2</v>
       </c>
       <c r="J48" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.73046875</v>
       </c>
       <c r="K48" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.26953125</v>
       </c>
     </row>
@@ -23046,23 +23130,23 @@
         <v>1442508</v>
       </c>
       <c r="G49" s="26">
+        <f t="shared" si="18"/>
+        <v>2.140625</v>
+      </c>
+      <c r="H49" s="26">
         <f t="shared" si="15"/>
-        <v>2.140625</v>
-      </c>
-      <c r="H49" s="26">
-        <f>(E49-$B49)/1024</f>
         <v>1.95703125</v>
       </c>
       <c r="I49" s="26">
-        <f>(D49-$B49)/1024</f>
+        <f t="shared" si="16"/>
         <v>1.9765625</v>
       </c>
       <c r="J49" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.78125</v>
       </c>
       <c r="K49" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.1953125</v>
       </c>
     </row>
@@ -23070,35 +23154,35 @@
       <c r="A50" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B50" s="69">
+      <c r="B50" s="66">
         <v>23940</v>
       </c>
-      <c r="C50" s="69">
+      <c r="C50" s="66">
         <v>25680</v>
       </c>
-      <c r="D50" s="69">
+      <c r="D50" s="66">
         <v>25684</v>
       </c>
-      <c r="E50" s="69">
+      <c r="E50" s="66">
         <v>25656</v>
       </c>
-      <c r="F50" s="69">
+      <c r="F50" s="66">
         <v>25664</v>
       </c>
-      <c r="G50" s="70">
-        <f t="shared" ref="G50" si="17">(C50-$B50)/1024</f>
+      <c r="G50" s="67">
+        <f t="shared" ref="G50" si="20">(C50-$B50)/1024</f>
         <v>1.69921875</v>
       </c>
-      <c r="H50" s="70">
-        <f>(E50-$B50)/1024</f>
+      <c r="H50" s="67">
+        <f t="shared" si="15"/>
         <v>1.67578125</v>
       </c>
-      <c r="I50" s="70">
-        <f>(D50-$B50)/1024</f>
+      <c r="I50" s="67">
+        <f t="shared" si="16"/>
         <v>1.703125</v>
       </c>
-      <c r="J50" s="70">
-        <f t="shared" ref="J50" si="18">(F50-$B50)/1024</f>
+      <c r="J50" s="67">
+        <f t="shared" ref="J50" si="21">(F50-$B50)/1024</f>
         <v>1.68359375</v>
       </c>
       <c r="K50" s="25"/>
@@ -23123,23 +23207,23 @@
         <v>8488</v>
       </c>
       <c r="G51" s="26">
+        <f t="shared" si="18"/>
+        <v>1.9453125</v>
+      </c>
+      <c r="H51" s="26">
         <f t="shared" si="15"/>
-        <v>1.9453125</v>
-      </c>
-      <c r="H51" s="26">
-        <f>(E51-$B51)/1024</f>
         <v>1.78125</v>
       </c>
       <c r="I51" s="26">
-        <f>(D51-$B51)/1024</f>
+        <f t="shared" si="16"/>
         <v>1.98046875</v>
       </c>
       <c r="J51" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.73828125</v>
       </c>
       <c r="K51" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.2421875</v>
       </c>
     </row>
@@ -23163,23 +23247,23 @@
         <v>7320</v>
       </c>
       <c r="G52" s="26">
+        <f t="shared" si="18"/>
+        <v>2.0234375</v>
+      </c>
+      <c r="H52" s="26">
         <f t="shared" si="15"/>
-        <v>2.0234375</v>
-      </c>
-      <c r="H52" s="26">
-        <f>(E52-$B52)/1024</f>
         <v>1.890625</v>
       </c>
       <c r="I52" s="26">
-        <f>(D52-$B52)/1024</f>
+        <f t="shared" si="16"/>
         <v>2.03515625</v>
       </c>
       <c r="J52" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.76953125</v>
       </c>
       <c r="K52" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0.265625</v>
       </c>
     </row>

</xml_diff>

<commit_message>
59 experiment persistent encoding vs non persistent encoding (#61)
* issue 59

* report for issue 59 (week 09)

* update weekly report
</commit_message>
<xml_diff>
--- a/docs/experiments.xlsx
+++ b/docs/experiments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sungkeunkim/git/DCCE/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A9233E-F441-B740-98A3-978DA6FE5C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DCE9DB-4FA3-264F-B842-014126C87E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{E6A628A0-BA48-FD4D-9B0A-CC4CBF8BF1CD}"/>
+    <workbookView xWindow="-75820" yWindow="-7700" windowWidth="38400" windowHeight="19700" firstSheet="3" activeTab="9" xr2:uid="{E6A628A0-BA48-FD4D-9B0A-CC4CBF8BF1CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench status" sheetId="11" r:id="rId1"/>
@@ -22,9 +22,31 @@
     <sheet name="Sheet1" sheetId="24" r:id="rId7"/>
     <sheet name="Dyn_Overhead_Splash3-analysis" sheetId="25" r:id="rId8"/>
     <sheet name="Sheet3" sheetId="26" r:id="rId9"/>
+    <sheet name="barrier-elision-dynamic" sheetId="28" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bench status'!$A$1:$I$58</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">'barrier-elision-dynamic'!$A$1:$B$32</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'barrier-elision-dynamic'!$H$2:$I$15</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'barrier-elision-dynamic'!$J$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'barrier-elision-dynamic'!$J$2:$J$15</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'barrier-elision-dynamic'!$K$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'barrier-elision-dynamic'!$K$2:$K$15</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'barrier-elision-dynamic'!$L$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">'barrier-elision-dynamic'!$L$2:$L$15</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">'barrier-elision-dynamic'!$M$1</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">'barrier-elision-dynamic'!$M$2:$M$15</definedName>
+    <definedName name="_xlchart.v2.10" hidden="1">'barrier-elision-dynamic'!$H$2:$H$15</definedName>
+    <definedName name="_xlchart.v2.11" hidden="1">'barrier-elision-dynamic'!$I$1</definedName>
+    <definedName name="_xlchart.v2.12" hidden="1">'barrier-elision-dynamic'!$I$2:$I$15</definedName>
+    <definedName name="_xlchart.v2.13" hidden="1">'barrier-elision-dynamic'!$J$1</definedName>
+    <definedName name="_xlchart.v2.14" hidden="1">'barrier-elision-dynamic'!$J$2:$J$15</definedName>
+    <definedName name="_xlchart.v2.15" hidden="1">'barrier-elision-dynamic'!$K$1</definedName>
+    <definedName name="_xlchart.v2.16" hidden="1">'barrier-elision-dynamic'!$K$2:$K$15</definedName>
+    <definedName name="_xlchart.v2.17" hidden="1">'barrier-elision-dynamic'!$L$1</definedName>
+    <definedName name="_xlchart.v2.18" hidden="1">'barrier-elision-dynamic'!$L$2:$L$15</definedName>
+    <definedName name="_xlchart.v2.19" hidden="1">'barrier-elision-dynamic'!$M$1</definedName>
+    <definedName name="_xlchart.v2.20" hidden="1">'barrier-elision-dynamic'!$M$2:$M$15</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -81,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="167">
   <si>
     <t>mcf_s</t>
   </si>
@@ -566,6 +588,24 @@
   <si>
     <t>GEOMEAN</t>
   </si>
+  <si>
+    <t>DCCE</t>
+  </si>
+  <si>
+    <t>DrCCTLib</t>
+  </si>
+  <si>
+    <t>Speedup</t>
+  </si>
+  <si>
+    <t>Number of Barrier Calls</t>
+  </si>
+  <si>
+    <t>Time for barrier call (ms)</t>
+  </si>
+  <si>
+    <t>% in total execution</t>
+  </si>
 </sst>
 </file>
 
@@ -689,7 +729,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -791,13 +831,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -881,6 +932,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -11413,6 +11471,851 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14771222969511"/>
+          <c:y val="0.16209609215514728"/>
+          <c:w val="0.84468068982763012"/>
+          <c:h val="0.42963242441916982"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$I$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Native</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="bg2">
+                <a:lumMod val="90000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$H$2:$H$15</c:f>
+              <c:strCache>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>701.BARNES</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>702.CHOLESKY</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>703.FFT</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>704.FMM</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>705.LU-CB</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>706.LU-NCB</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>707.OCEAN-CP</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>708.OCEAN-NCP</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>709.RADIOSITY</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>710.RADIX</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>711.RAYTRACE</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>713.WATER-NSQUARED</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>714.WATER-SPATIAL</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>goemean</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'barrier-elision-dynamic'!$I$2:$I$15</c:f>
+              <c:numCache>
+                <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-EA6F-0D40-931C-5646C6A86955}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Empty client</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="bg2">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$H$2:$H$15</c:f>
+              <c:strCache>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>701.BARNES</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>702.CHOLESKY</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>703.FFT</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>704.FMM</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>705.LU-CB</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>706.LU-NCB</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>707.OCEAN-CP</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>708.OCEAN-NCP</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>709.RADIOSITY</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>710.RADIX</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>711.RAYTRACE</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>713.WATER-NSQUARED</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>714.WATER-SPATIAL</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>goemean</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'barrier-elision-dynamic'!$J$2:$J$15</c:f>
+              <c:numCache>
+                <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>1.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.3636363636363635</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5293288708825084</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.2195121951219512</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.0377295492487479</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0470823941898322</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.0883816213052384</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.95233142659039693</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.3793103448275863</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0706467661691543</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.2215416028586012</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.1012931034482758</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.4615384615384615</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.207830443650467</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-EA6F-0D40-931C-5646C6A86955}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$K$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>DCCE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$H$2:$H$15</c:f>
+              <c:strCache>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>701.BARNES</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>702.CHOLESKY</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>703.FFT</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>704.FMM</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>705.LU-CB</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>706.LU-NCB</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>707.OCEAN-CP</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>708.OCEAN-NCP</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>709.RADIOSITY</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>710.RADIX</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>711.RAYTRACE</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>713.WATER-NSQUARED</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>714.WATER-SPATIAL</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>goemean</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'barrier-elision-dynamic'!$K$2:$K$15</c:f>
+              <c:numCache>
+                <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>12.55</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.8636363636363638</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.7646644354412544</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.1707317073170733</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.9288814691151916</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.1277235161532682</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.2250512145156569</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.95510487086150109</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>12.206896551724139</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.9293532338308457</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10.118938233792752</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.3232758620689653</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6.0384615384615383</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.2225007715773319</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-EA6F-0D40-931C-5646C6A86955}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$L$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>DrCCTLib</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'barrier-elision-dynamic'!$H$2:$H$15</c:f>
+              <c:strCache>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>701.BARNES</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>702.CHOLESKY</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>703.FFT</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>704.FMM</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>705.LU-CB</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>706.LU-NCB</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>707.OCEAN-CP</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>708.OCEAN-NCP</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>709.RADIOSITY</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>710.RADIX</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>711.RAYTRACE</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>713.WATER-NSQUARED</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>714.WATER-SPATIAL</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>goemean</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'barrier-elision-dynamic'!$L$2:$L$15</c:f>
+              <c:numCache>
+                <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>19.649999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.3655099524396697</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.975609756097561</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.1445742904841403</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.8690207863761579</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.2780216564237636</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.0570289478245796</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>18.413793103448278</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.5562189054726367</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>14.344053088310362</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.0107758620689653</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>7.8461538461538458</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.5819772016716263</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-EA6F-0D40-931C-5646C6A86955}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="575708623"/>
+        <c:axId val="575805615"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="575708623"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="3600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Tw Cen MT" panose="020B0602020104020603" pitchFamily="34" charset="77"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="575805615"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="575805615"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="20"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="3600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="Tw Cen MT" panose="020B0602020104020603" pitchFamily="34" charset="77"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Runtime Overhead</a:t>
+                </a:r>
+              </a:p>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Relative to Native (times)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="3600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Tw Cen MT" panose="020B0602020104020603" pitchFamily="34" charset="77"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="3600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Tw Cen MT" panose="020B0602020104020603" pitchFamily="34" charset="77"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="575708623"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="2"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13980485837707787"/>
+          <c:y val="2.7520851560221639E-2"/>
+          <c:w val="0.84838678368328957"/>
+          <c:h val="0.1193791921843103"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="3200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="Tw Cen MT" panose="020B0602020104020603" pitchFamily="34" charset="77"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="3600">
+          <a:latin typeface="Tw Cen MT" panose="020B0602020104020603" pitchFamily="34" charset="77"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -11694,6 +12597,46 @@
 </file>
 
 <file path=xl/charts/colors8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -15757,6 +16700,509 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -16086,6 +17532,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1333500</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{442B353D-09C4-7B49-988B-40B0B5C50834}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -17917,6 +19406,1117 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5B47E61-5499-7241-8D93-4870A5537F5A}">
+  <dimension ref="A1:X32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="9.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="13" width="9.83203125" customWidth="1"/>
+    <col min="14" max="17" width="9.6640625" customWidth="1"/>
+    <col min="19" max="24" width="25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E1" s="71" t="s">
+        <v>162</v>
+      </c>
+      <c r="F1" s="71"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="L1" s="72" t="s">
+        <v>162</v>
+      </c>
+      <c r="M1" s="72" t="s">
+        <v>163</v>
+      </c>
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="76"/>
+      <c r="Q1" s="76"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="W1" s="75"/>
+    </row>
+    <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="3">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3">
+        <v>28</v>
+      </c>
+      <c r="D2" s="3">
+        <v>251</v>
+      </c>
+      <c r="E2" s="3">
+        <v>393</v>
+      </c>
+      <c r="F2" s="20"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" s="20">
+        <f>B2/$B2</f>
+        <v>1</v>
+      </c>
+      <c r="J2" s="20">
+        <f>C2/$B2</f>
+        <v>1.4</v>
+      </c>
+      <c r="K2" s="20">
+        <f>D2/$B2</f>
+        <v>12.55</v>
+      </c>
+      <c r="L2" s="20">
+        <f>E2/$B2</f>
+        <v>19.649999999999999</v>
+      </c>
+      <c r="M2" s="73">
+        <f>L2/K2</f>
+        <v>1.5657370517928284</v>
+      </c>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="X2" s="72" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="3">
+        <v>22</v>
+      </c>
+      <c r="C3" s="3">
+        <v>30</v>
+      </c>
+      <c r="D3" s="3">
+        <v>63</v>
+      </c>
+      <c r="E3" s="3">
+        <v>88</v>
+      </c>
+      <c r="F3" s="20"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="20">
+        <f>B3/$B3</f>
+        <v>1</v>
+      </c>
+      <c r="J3" s="20">
+        <f>C3/$B3</f>
+        <v>1.3636363636363635</v>
+      </c>
+      <c r="K3" s="20">
+        <f>D3/$B3</f>
+        <v>2.8636363636363638</v>
+      </c>
+      <c r="L3" s="20">
+        <f>E3/$B3</f>
+        <v>4</v>
+      </c>
+      <c r="M3" s="73">
+        <f t="shared" ref="M3:M15" si="0">L3/K3</f>
+        <v>1.3968253968253967</v>
+      </c>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="S3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="T3" s="3">
+        <v>34</v>
+      </c>
+      <c r="U3" s="3">
+        <v>0</v>
+      </c>
+      <c r="V3" s="3">
+        <v>34</v>
+      </c>
+      <c r="W3" s="3">
+        <v>9</v>
+      </c>
+      <c r="X3" s="8"/>
+    </row>
+    <row r="4" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="3">
+        <v>5677</v>
+      </c>
+      <c r="C4" s="3">
+        <v>8682</v>
+      </c>
+      <c r="D4" s="3">
+        <v>32726</v>
+      </c>
+      <c r="E4" s="3">
+        <v>53168</v>
+      </c>
+      <c r="F4" s="20"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="20">
+        <f>B4/$B4</f>
+        <v>1</v>
+      </c>
+      <c r="J4" s="20">
+        <f>C4/$B4</f>
+        <v>1.5293288708825084</v>
+      </c>
+      <c r="K4" s="20">
+        <f>D4/$B4</f>
+        <v>5.7646644354412544</v>
+      </c>
+      <c r="L4" s="20">
+        <f>E4/$B4</f>
+        <v>9.3655099524396697</v>
+      </c>
+      <c r="M4" s="73">
+        <f t="shared" si="0"/>
+        <v>1.6246409582594878</v>
+      </c>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="S4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="T4" s="3">
+        <v>8</v>
+      </c>
+      <c r="U4" s="3">
+        <v>0</v>
+      </c>
+      <c r="V4" s="3">
+        <v>8</v>
+      </c>
+      <c r="W4" s="3">
+        <v>4</v>
+      </c>
+      <c r="X4" s="8"/>
+    </row>
+    <row r="5" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="3">
+        <v>41</v>
+      </c>
+      <c r="C5" s="3">
+        <v>50</v>
+      </c>
+      <c r="D5" s="3">
+        <v>89</v>
+      </c>
+      <c r="E5" s="3">
+        <v>122</v>
+      </c>
+      <c r="F5" s="20"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="I5" s="20">
+        <f>B5/$B5</f>
+        <v>1</v>
+      </c>
+      <c r="J5" s="20">
+        <f>C5/$B5</f>
+        <v>1.2195121951219512</v>
+      </c>
+      <c r="K5" s="20">
+        <f>D5/$B5</f>
+        <v>2.1707317073170733</v>
+      </c>
+      <c r="L5" s="20">
+        <f>E5/$B5</f>
+        <v>2.975609756097561</v>
+      </c>
+      <c r="M5" s="73">
+        <f t="shared" si="0"/>
+        <v>1.3707865168539324</v>
+      </c>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="S5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="T5" s="3">
+        <v>14</v>
+      </c>
+      <c r="U5" s="3">
+        <v>0</v>
+      </c>
+      <c r="V5" s="3">
+        <v>14</v>
+      </c>
+      <c r="W5" s="3">
+        <v>5</v>
+      </c>
+      <c r="X5" s="8"/>
+    </row>
+    <row r="6" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2995</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3108</v>
+      </c>
+      <c r="D6" s="3">
+        <v>14762</v>
+      </c>
+      <c r="E6" s="3">
+        <v>18403</v>
+      </c>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I6" s="20">
+        <f>B6/$B6</f>
+        <v>1</v>
+      </c>
+      <c r="J6" s="20">
+        <f>C6/$B6</f>
+        <v>1.0377295492487479</v>
+      </c>
+      <c r="K6" s="20">
+        <f>D6/$B6</f>
+        <v>4.9288814691151916</v>
+      </c>
+      <c r="L6" s="20">
+        <f>E6/$B6</f>
+        <v>6.1445742904841403</v>
+      </c>
+      <c r="M6" s="73">
+        <f t="shared" si="0"/>
+        <v>1.2466467958271239</v>
+      </c>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="S6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T6" s="3">
+        <v>68</v>
+      </c>
+      <c r="U6" s="3">
+        <v>0</v>
+      </c>
+      <c r="V6" s="3">
+        <v>68</v>
+      </c>
+      <c r="W6" s="3">
+        <v>26</v>
+      </c>
+      <c r="X6" s="8"/>
+    </row>
+    <row r="7" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="3">
+        <v>3993</v>
+      </c>
+      <c r="C7" s="3">
+        <v>4181</v>
+      </c>
+      <c r="D7" s="3">
+        <v>16482</v>
+      </c>
+      <c r="E7" s="3">
+        <v>19442</v>
+      </c>
+      <c r="F7" s="20"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" s="20">
+        <f>B7/$B7</f>
+        <v>1</v>
+      </c>
+      <c r="J7" s="20">
+        <f>C7/$B7</f>
+        <v>1.0470823941898322</v>
+      </c>
+      <c r="K7" s="20">
+        <f>D7/$B7</f>
+        <v>4.1277235161532682</v>
+      </c>
+      <c r="L7" s="20">
+        <f>E7/$B7</f>
+        <v>4.8690207863761579</v>
+      </c>
+      <c r="M7" s="73">
+        <f t="shared" si="0"/>
+        <v>1.1795898556000484</v>
+      </c>
+      <c r="N7" s="21"/>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="S7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="T7" s="3">
+        <v>1030</v>
+      </c>
+      <c r="U7" s="3">
+        <v>0</v>
+      </c>
+      <c r="V7" s="3">
+        <v>1030</v>
+      </c>
+      <c r="W7" s="3">
+        <v>524</v>
+      </c>
+      <c r="X7" s="8"/>
+    </row>
+    <row r="8" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3417</v>
+      </c>
+      <c r="C8" s="3">
+        <v>3719</v>
+      </c>
+      <c r="D8" s="3">
+        <v>4186</v>
+      </c>
+      <c r="E8" s="3">
+        <v>4367</v>
+      </c>
+      <c r="F8" s="20"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I8" s="20">
+        <f>B8/$B8</f>
+        <v>1</v>
+      </c>
+      <c r="J8" s="20">
+        <f>C8/$B8</f>
+        <v>1.0883816213052384</v>
+      </c>
+      <c r="K8" s="20">
+        <f>D8/$B8</f>
+        <v>1.2250512145156569</v>
+      </c>
+      <c r="L8" s="20">
+        <f>E8/$B8</f>
+        <v>1.2780216564237636</v>
+      </c>
+      <c r="M8" s="73">
+        <f t="shared" si="0"/>
+        <v>1.043239369326326</v>
+      </c>
+      <c r="N8" s="21"/>
+      <c r="O8" s="21"/>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="S8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="T8" s="3">
+        <v>1030</v>
+      </c>
+      <c r="U8" s="3">
+        <v>1</v>
+      </c>
+      <c r="V8" s="3">
+        <v>1030</v>
+      </c>
+      <c r="W8" s="3">
+        <v>431</v>
+      </c>
+      <c r="X8" s="8"/>
+    </row>
+    <row r="9" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="3">
+        <v>5769</v>
+      </c>
+      <c r="C9" s="3">
+        <v>5494</v>
+      </c>
+      <c r="D9" s="3">
+        <v>5510</v>
+      </c>
+      <c r="E9" s="3">
+        <v>6098</v>
+      </c>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I9" s="20">
+        <f>B9/$B9</f>
+        <v>1</v>
+      </c>
+      <c r="J9" s="20">
+        <f>C9/$B9</f>
+        <v>0.95233142659039693</v>
+      </c>
+      <c r="K9" s="20">
+        <f>D9/$B9</f>
+        <v>0.95510487086150109</v>
+      </c>
+      <c r="L9" s="20">
+        <f>E9/$B9</f>
+        <v>1.0570289478245796</v>
+      </c>
+      <c r="M9" s="73">
+        <f t="shared" si="0"/>
+        <v>1.1067150635208711</v>
+      </c>
+      <c r="N9" s="21"/>
+      <c r="O9" s="21"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="S9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="T9" s="3">
+        <v>1336</v>
+      </c>
+      <c r="U9" s="3">
+        <v>0</v>
+      </c>
+      <c r="V9" s="3">
+        <v>1336</v>
+      </c>
+      <c r="W9" s="3">
+        <v>1047</v>
+      </c>
+      <c r="X9" s="8"/>
+    </row>
+    <row r="10" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="3">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3">
+        <v>40</v>
+      </c>
+      <c r="D10" s="3">
+        <v>354</v>
+      </c>
+      <c r="E10" s="3">
+        <v>534</v>
+      </c>
+      <c r="F10" s="20"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="I10" s="20">
+        <f>B10/$B10</f>
+        <v>1</v>
+      </c>
+      <c r="J10" s="20">
+        <f>C10/$B10</f>
+        <v>1.3793103448275863</v>
+      </c>
+      <c r="K10" s="20">
+        <f>D10/$B10</f>
+        <v>12.206896551724139</v>
+      </c>
+      <c r="L10" s="20">
+        <f>E10/$B10</f>
+        <v>18.413793103448278</v>
+      </c>
+      <c r="M10" s="73">
+        <f t="shared" si="0"/>
+        <v>1.5084745762711864</v>
+      </c>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="S10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="T10" s="3">
+        <v>1300</v>
+      </c>
+      <c r="U10" s="3">
+        <v>0</v>
+      </c>
+      <c r="V10" s="3">
+        <v>1300</v>
+      </c>
+      <c r="W10" s="3">
+        <v>844</v>
+      </c>
+      <c r="X10" s="8"/>
+    </row>
+    <row r="11" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A11" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="3">
+        <v>1005</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1076</v>
+      </c>
+      <c r="D11" s="3">
+        <v>3949</v>
+      </c>
+      <c r="E11" s="3">
+        <v>5584</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="20">
+        <f>B11/$B11</f>
+        <v>1</v>
+      </c>
+      <c r="J11" s="20">
+        <f>C11/$B11</f>
+        <v>1.0706467661691543</v>
+      </c>
+      <c r="K11" s="20">
+        <f>D11/$B11</f>
+        <v>3.9293532338308457</v>
+      </c>
+      <c r="L11" s="20">
+        <f>E11/$B11</f>
+        <v>5.5562189054726367</v>
+      </c>
+      <c r="M11" s="73">
+        <f t="shared" si="0"/>
+        <v>1.4140288680678652</v>
+      </c>
+      <c r="N11" s="21"/>
+      <c r="O11" s="21"/>
+      <c r="P11" s="21"/>
+      <c r="Q11" s="21"/>
+      <c r="S11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="T11" s="3">
+        <v>20</v>
+      </c>
+      <c r="U11" s="3">
+        <v>0</v>
+      </c>
+      <c r="V11" s="3">
+        <v>20</v>
+      </c>
+      <c r="W11" s="3">
+        <v>12</v>
+      </c>
+      <c r="X11" s="8"/>
+    </row>
+    <row r="12" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A12" s="74" t="s">
+        <v>154</v>
+      </c>
+      <c r="B12" s="3">
+        <v>5877</v>
+      </c>
+      <c r="C12" s="3">
+        <v>7179</v>
+      </c>
+      <c r="D12" s="3">
+        <v>59469</v>
+      </c>
+      <c r="E12" s="3">
+        <v>84300</v>
+      </c>
+      <c r="F12" s="20"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="74" t="s">
+        <v>154</v>
+      </c>
+      <c r="I12" s="20">
+        <f>B12/$B12</f>
+        <v>1</v>
+      </c>
+      <c r="J12" s="20">
+        <f>C12/$B12</f>
+        <v>1.2215416028586012</v>
+      </c>
+      <c r="K12" s="20">
+        <f>D12/$B12</f>
+        <v>10.118938233792752</v>
+      </c>
+      <c r="L12" s="20">
+        <f>E12/$B12</f>
+        <v>14.344053088310362</v>
+      </c>
+      <c r="M12" s="73">
+        <f t="shared" si="0"/>
+        <v>1.417545275689855</v>
+      </c>
+      <c r="N12" s="21"/>
+      <c r="O12" s="21"/>
+      <c r="P12" s="21"/>
+      <c r="Q12" s="21"/>
+      <c r="S12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="T12" s="3">
+        <v>30</v>
+      </c>
+      <c r="U12" s="3">
+        <v>0</v>
+      </c>
+      <c r="V12" s="3">
+        <v>30</v>
+      </c>
+      <c r="W12" s="3">
+        <v>12</v>
+      </c>
+      <c r="X12" s="8"/>
+    </row>
+    <row r="13" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="3">
+        <v>464</v>
+      </c>
+      <c r="C13" s="3">
+        <v>511</v>
+      </c>
+      <c r="D13" s="3">
+        <v>2006</v>
+      </c>
+      <c r="E13" s="3">
+        <v>2325</v>
+      </c>
+      <c r="F13" s="20"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I13" s="20">
+        <f>B13/$B13</f>
+        <v>1</v>
+      </c>
+      <c r="J13" s="20">
+        <f>C13/$B13</f>
+        <v>1.1012931034482758</v>
+      </c>
+      <c r="K13" s="20">
+        <f>D13/$B13</f>
+        <v>4.3232758620689653</v>
+      </c>
+      <c r="L13" s="20">
+        <f>E13/$B13</f>
+        <v>5.0107758620689653</v>
+      </c>
+      <c r="M13" s="73">
+        <f t="shared" si="0"/>
+        <v>1.1590229312063809</v>
+      </c>
+      <c r="N13" s="21"/>
+      <c r="O13" s="21"/>
+      <c r="P13" s="21"/>
+      <c r="Q13" s="21"/>
+      <c r="S13" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="T13" s="3">
+        <v>2</v>
+      </c>
+      <c r="U13" s="3">
+        <v>0</v>
+      </c>
+      <c r="V13" s="3">
+        <v>2</v>
+      </c>
+      <c r="W13" s="3">
+        <v>1</v>
+      </c>
+      <c r="X13" s="8"/>
+    </row>
+    <row r="14" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="3">
+        <v>52</v>
+      </c>
+      <c r="C14" s="3">
+        <v>76</v>
+      </c>
+      <c r="D14" s="3">
+        <v>314</v>
+      </c>
+      <c r="E14" s="3">
+        <v>408</v>
+      </c>
+      <c r="F14" s="20"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" s="20">
+        <f>B14/$B14</f>
+        <v>1</v>
+      </c>
+      <c r="J14" s="20">
+        <f>C14/$B14</f>
+        <v>1.4615384615384615</v>
+      </c>
+      <c r="K14" s="20">
+        <f>D14/$B14</f>
+        <v>6.0384615384615383</v>
+      </c>
+      <c r="L14" s="20">
+        <f>E14/$B14</f>
+        <v>7.8461538461538458</v>
+      </c>
+      <c r="M14" s="73">
+        <f t="shared" si="0"/>
+        <v>1.2993630573248407</v>
+      </c>
+      <c r="N14" s="21"/>
+      <c r="O14" s="21"/>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="21"/>
+      <c r="S14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="T14" s="3">
+        <v>50</v>
+      </c>
+      <c r="U14" s="3">
+        <v>0</v>
+      </c>
+      <c r="V14" s="3">
+        <v>50</v>
+      </c>
+      <c r="W14" s="3">
+        <v>17</v>
+      </c>
+      <c r="X14" s="8"/>
+    </row>
+    <row r="15" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="H15" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I15" s="20">
+        <f>GEOMEAN(I2:I14)</f>
+        <v>1</v>
+      </c>
+      <c r="J15" s="20">
+        <f>GEOMEAN(J2:J14)</f>
+        <v>1.207830443650467</v>
+      </c>
+      <c r="K15" s="20">
+        <f>GEOMEAN(K2:K14)</f>
+        <v>4.2225007715773319</v>
+      </c>
+      <c r="L15" s="20">
+        <f>GEOMEAN(L2:L14)</f>
+        <v>5.5819772016716263</v>
+      </c>
+      <c r="M15" s="73">
+        <f t="shared" si="0"/>
+        <v>1.3219600193433372</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="T15" s="3">
+        <v>40</v>
+      </c>
+      <c r="U15" s="3">
+        <v>0</v>
+      </c>
+      <c r="V15" s="3">
+        <v>40</v>
+      </c>
+      <c r="W15" s="3">
+        <v>12</v>
+      </c>
+      <c r="X15" s="8"/>
+    </row>
+    <row r="18" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G18" s="76"/>
+      <c r="H18" s="76"/>
+      <c r="I18" s="76"/>
+      <c r="J18" s="76"/>
+      <c r="K18" s="76"/>
+      <c r="L18" s="76"/>
+      <c r="M18" s="76"/>
+      <c r="N18" s="76"/>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="76"/>
+    </row>
+    <row r="19" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G19" s="77"/>
+      <c r="H19" s="77"/>
+      <c r="I19" s="77"/>
+      <c r="J19" s="77"/>
+      <c r="K19" s="77"/>
+      <c r="L19" s="77"/>
+      <c r="M19" s="77"/>
+      <c r="N19" s="77"/>
+      <c r="O19" s="77"/>
+      <c r="P19" s="77"/>
+      <c r="Q19" s="77"/>
+    </row>
+    <row r="20" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="77"/>
+      <c r="J20" s="77"/>
+      <c r="K20" s="77"/>
+      <c r="L20" s="77"/>
+      <c r="M20" s="77"/>
+      <c r="N20" s="77"/>
+      <c r="O20" s="77"/>
+      <c r="P20" s="77"/>
+      <c r="Q20" s="77"/>
+    </row>
+    <row r="21" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G21" s="77"/>
+      <c r="H21" s="77"/>
+      <c r="I21" s="77"/>
+      <c r="J21" s="77"/>
+      <c r="K21" s="77"/>
+      <c r="L21" s="77"/>
+      <c r="M21" s="77"/>
+      <c r="N21" s="77"/>
+      <c r="O21" s="77"/>
+      <c r="P21" s="77"/>
+      <c r="Q21" s="77"/>
+    </row>
+    <row r="22" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="77"/>
+      <c r="K22" s="77"/>
+      <c r="L22" s="77"/>
+      <c r="M22" s="77"/>
+      <c r="N22" s="77"/>
+      <c r="O22" s="77"/>
+      <c r="P22" s="77"/>
+      <c r="Q22" s="77"/>
+    </row>
+    <row r="23" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G23" s="77"/>
+      <c r="H23" s="77"/>
+      <c r="I23" s="77"/>
+      <c r="J23" s="77"/>
+      <c r="K23" s="77"/>
+      <c r="L23" s="77"/>
+      <c r="M23" s="77"/>
+      <c r="N23" s="77"/>
+      <c r="O23" s="77"/>
+      <c r="P23" s="77"/>
+      <c r="Q23" s="77"/>
+    </row>
+    <row r="24" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G24" s="77"/>
+      <c r="H24" s="77"/>
+      <c r="I24" s="77"/>
+      <c r="J24" s="77"/>
+      <c r="K24" s="77"/>
+      <c r="L24" s="77"/>
+      <c r="M24" s="77"/>
+      <c r="N24" s="77"/>
+      <c r="O24" s="77"/>
+      <c r="P24" s="77"/>
+      <c r="Q24" s="77"/>
+    </row>
+    <row r="25" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G25" s="77"/>
+      <c r="H25" s="77"/>
+      <c r="I25" s="77"/>
+      <c r="J25" s="77"/>
+      <c r="K25" s="77"/>
+      <c r="L25" s="77"/>
+      <c r="M25" s="77"/>
+      <c r="N25" s="77"/>
+      <c r="O25" s="77"/>
+      <c r="P25" s="77"/>
+      <c r="Q25" s="77"/>
+    </row>
+    <row r="26" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G26" s="77"/>
+      <c r="H26" s="77"/>
+      <c r="I26" s="77"/>
+      <c r="J26" s="77"/>
+      <c r="K26" s="77"/>
+      <c r="L26" s="77"/>
+      <c r="M26" s="77"/>
+      <c r="N26" s="77"/>
+      <c r="O26" s="77"/>
+      <c r="P26" s="77"/>
+      <c r="Q26" s="77"/>
+    </row>
+    <row r="27" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G27" s="77"/>
+      <c r="H27" s="77"/>
+      <c r="I27" s="77"/>
+      <c r="J27" s="77"/>
+      <c r="K27" s="77"/>
+      <c r="L27" s="77"/>
+      <c r="M27" s="77"/>
+      <c r="N27" s="77"/>
+      <c r="O27" s="77"/>
+      <c r="P27" s="77"/>
+      <c r="Q27" s="77"/>
+    </row>
+    <row r="28" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G28" s="77"/>
+      <c r="H28" s="77"/>
+      <c r="I28" s="77"/>
+      <c r="J28" s="77"/>
+      <c r="K28" s="77"/>
+      <c r="L28" s="77"/>
+      <c r="M28" s="77"/>
+      <c r="N28" s="77"/>
+      <c r="O28" s="77"/>
+      <c r="P28" s="77"/>
+      <c r="Q28" s="77"/>
+    </row>
+    <row r="29" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G29" s="77"/>
+      <c r="H29" s="77"/>
+      <c r="I29" s="77"/>
+      <c r="J29" s="77"/>
+      <c r="K29" s="77"/>
+      <c r="L29" s="77"/>
+      <c r="M29" s="77"/>
+      <c r="N29" s="77"/>
+      <c r="O29" s="77"/>
+      <c r="P29" s="77"/>
+      <c r="Q29" s="77"/>
+    </row>
+    <row r="30" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G30" s="77"/>
+      <c r="H30" s="77"/>
+      <c r="I30" s="77"/>
+      <c r="J30" s="77"/>
+      <c r="K30" s="77"/>
+      <c r="L30" s="77"/>
+      <c r="M30" s="77"/>
+      <c r="N30" s="77"/>
+      <c r="O30" s="77"/>
+      <c r="P30" s="77"/>
+      <c r="Q30" s="77"/>
+    </row>
+    <row r="31" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G31" s="77"/>
+      <c r="H31" s="77"/>
+      <c r="I31" s="77"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="77"/>
+      <c r="L31" s="77"/>
+      <c r="M31" s="77"/>
+      <c r="N31" s="77"/>
+      <c r="O31" s="77"/>
+      <c r="P31" s="77"/>
+      <c r="Q31" s="77"/>
+    </row>
+    <row r="32" spans="7:17" ht="18" x14ac:dyDescent="0.2">
+      <c r="G32" s="77"/>
+      <c r="H32" s="77"/>
+      <c r="I32" s="77"/>
+      <c r="J32" s="77"/>
+      <c r="K32" s="77"/>
+      <c r="L32" s="77"/>
+      <c r="M32" s="77"/>
+      <c r="N32" s="77"/>
+      <c r="O32" s="77"/>
+      <c r="P32" s="77"/>
+      <c r="Q32" s="77"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BF8609-3905-414C-9DEE-F349E5DBD3B1}">
   <dimension ref="B1:Q117"/>

</xml_diff>

<commit_message>
59 experiment persistent encoding vs non persistent encoding (#62)
* issue 59

* report for issue 59 (week 09)

* update weekly report

* update docs
</commit_message>
<xml_diff>
--- a/docs/experiments.xlsx
+++ b/docs/experiments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sungkeunkim/git/DCCE/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DCE9DB-4FA3-264F-B842-014126C87E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BBA804-6D7C-EF4F-B1F0-825C946EF0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-75820" yWindow="-7700" windowWidth="38400" windowHeight="19700" firstSheet="3" activeTab="9" xr2:uid="{E6A628A0-BA48-FD4D-9B0A-CC4CBF8BF1CD}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17480" firstSheet="3" activeTab="9" xr2:uid="{E6A628A0-BA48-FD4D-9B0A-CC4CBF8BF1CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench status" sheetId="11" r:id="rId1"/>
@@ -26,27 +26,6 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bench status'!$A$1:$I$58</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">'barrier-elision-dynamic'!$A$1:$B$32</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'barrier-elision-dynamic'!$H$2:$I$15</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'barrier-elision-dynamic'!$J$1</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'barrier-elision-dynamic'!$J$2:$J$15</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'barrier-elision-dynamic'!$K$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'barrier-elision-dynamic'!$K$2:$K$15</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'barrier-elision-dynamic'!$L$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'barrier-elision-dynamic'!$L$2:$L$15</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">'barrier-elision-dynamic'!$M$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'barrier-elision-dynamic'!$M$2:$M$15</definedName>
-    <definedName name="_xlchart.v2.10" hidden="1">'barrier-elision-dynamic'!$H$2:$H$15</definedName>
-    <definedName name="_xlchart.v2.11" hidden="1">'barrier-elision-dynamic'!$I$1</definedName>
-    <definedName name="_xlchart.v2.12" hidden="1">'barrier-elision-dynamic'!$I$2:$I$15</definedName>
-    <definedName name="_xlchart.v2.13" hidden="1">'barrier-elision-dynamic'!$J$1</definedName>
-    <definedName name="_xlchart.v2.14" hidden="1">'barrier-elision-dynamic'!$J$2:$J$15</definedName>
-    <definedName name="_xlchart.v2.15" hidden="1">'barrier-elision-dynamic'!$K$1</definedName>
-    <definedName name="_xlchart.v2.16" hidden="1">'barrier-elision-dynamic'!$K$2:$K$15</definedName>
-    <definedName name="_xlchart.v2.17" hidden="1">'barrier-elision-dynamic'!$L$1</definedName>
-    <definedName name="_xlchart.v2.18" hidden="1">'barrier-elision-dynamic'!$L$2:$L$15</definedName>
-    <definedName name="_xlchart.v2.19" hidden="1">'barrier-elision-dynamic'!$M$1</definedName>
-    <definedName name="_xlchart.v2.20" hidden="1">'barrier-elision-dynamic'!$M$2:$M$15</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -103,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="170">
   <si>
     <t>mcf_s</t>
   </si>
@@ -606,6 +585,15 @@
   <si>
     <t>% in total execution</t>
   </si>
+  <si>
+    <t>BE-DCCE</t>
+  </si>
+  <si>
+    <t>BE-DrCCTLib</t>
+  </si>
+  <si>
+    <t>BE-Empty client</t>
+  </si>
 </sst>
 </file>
 
@@ -848,7 +836,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -923,6 +911,10 @@
     <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -932,13 +924,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -11495,7 +11480,7 @@
           <c:x val="0.14771222969511"/>
           <c:y val="0.16209609215514728"/>
           <c:w val="0.84468068982763012"/>
-          <c:h val="0.42963242441916982"/>
+          <c:h val="0.43694237233503708"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -11646,7 +11631,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Empty client</c:v>
+                  <c:v>BE-Empty client</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -11781,7 +11766,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>DCCE</c:v>
+                  <c:v>BE-DCCE</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -11917,7 +11902,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>DrCCTLib</c:v>
+                  <c:v>BE-DrCCTLib</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -17536,16 +17521,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1333500</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>698500</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>520700</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -19432,11 +19417,11 @@
       <c r="D1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E1" s="71" t="s">
+      <c r="E1" s="68" t="s">
         <v>162</v>
       </c>
-      <c r="F1" s="71"/>
-      <c r="G1" s="76"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="1"/>
       <c r="H1" s="2" t="s">
         <v>87</v>
       </c>
@@ -19444,21 +19429,21 @@
         <v>86</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>104</v>
+        <v>169</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="L1" s="72" t="s">
-        <v>162</v>
-      </c>
-      <c r="M1" s="72" t="s">
+        <v>167</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
-      <c r="P1" s="76"/>
-      <c r="Q1" s="76"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2" t="s">
         <v>161</v>
@@ -19467,7 +19452,7 @@
       <c r="V1" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="W1" s="75"/>
+      <c r="W1" s="70"/>
     </row>
     <row r="2" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
@@ -19491,22 +19476,22 @@
         <v>69</v>
       </c>
       <c r="I2" s="20">
-        <f>B2/$B2</f>
+        <f t="shared" ref="I2:I14" si="0">B2/$B2</f>
         <v>1</v>
       </c>
       <c r="J2" s="20">
-        <f>C2/$B2</f>
+        <f t="shared" ref="J2:J14" si="1">C2/$B2</f>
         <v>1.4</v>
       </c>
       <c r="K2" s="20">
-        <f>D2/$B2</f>
+        <f t="shared" ref="K2:K14" si="2">D2/$B2</f>
         <v>12.55</v>
       </c>
       <c r="L2" s="20">
-        <f>E2/$B2</f>
+        <f t="shared" ref="L2:L14" si="3">E2/$B2</f>
         <v>19.649999999999999</v>
       </c>
-      <c r="M2" s="73">
+      <c r="M2" s="69">
         <f>L2/K2</f>
         <v>1.5657370517928284</v>
       </c>
@@ -19527,7 +19512,7 @@
       <c r="W2" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="X2" s="72" t="s">
+      <c r="X2" s="2" t="s">
         <v>166</v>
       </c>
     </row>
@@ -19553,23 +19538,23 @@
         <v>70</v>
       </c>
       <c r="I3" s="20">
-        <f>B3/$B3</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J3" s="20">
-        <f>C3/$B3</f>
+        <f t="shared" si="1"/>
         <v>1.3636363636363635</v>
       </c>
       <c r="K3" s="20">
-        <f>D3/$B3</f>
+        <f t="shared" si="2"/>
         <v>2.8636363636363638</v>
       </c>
       <c r="L3" s="20">
-        <f>E3/$B3</f>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="M3" s="73">
-        <f t="shared" ref="M3:M15" si="0">L3/K3</f>
+      <c r="M3" s="69">
+        <f t="shared" ref="M3:M15" si="4">L3/K3</f>
         <v>1.3968253968253967</v>
       </c>
       <c r="N3" s="21"/>
@@ -19615,23 +19600,23 @@
         <v>71</v>
       </c>
       <c r="I4" s="20">
-        <f>B4/$B4</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J4" s="20">
-        <f>C4/$B4</f>
+        <f t="shared" si="1"/>
         <v>1.5293288708825084</v>
       </c>
       <c r="K4" s="20">
-        <f>D4/$B4</f>
+        <f t="shared" si="2"/>
         <v>5.7646644354412544</v>
       </c>
       <c r="L4" s="20">
-        <f>E4/$B4</f>
+        <f t="shared" si="3"/>
         <v>9.3655099524396697</v>
       </c>
-      <c r="M4" s="73">
-        <f t="shared" si="0"/>
+      <c r="M4" s="69">
+        <f t="shared" si="4"/>
         <v>1.6246409582594878</v>
       </c>
       <c r="N4" s="21"/>
@@ -19677,23 +19662,23 @@
         <v>72</v>
       </c>
       <c r="I5" s="20">
-        <f>B5/$B5</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J5" s="20">
-        <f>C5/$B5</f>
+        <f t="shared" si="1"/>
         <v>1.2195121951219512</v>
       </c>
       <c r="K5" s="20">
-        <f>D5/$B5</f>
+        <f t="shared" si="2"/>
         <v>2.1707317073170733</v>
       </c>
       <c r="L5" s="20">
-        <f>E5/$B5</f>
+        <f t="shared" si="3"/>
         <v>2.975609756097561</v>
       </c>
-      <c r="M5" s="73">
-        <f t="shared" si="0"/>
+      <c r="M5" s="69">
+        <f t="shared" si="4"/>
         <v>1.3707865168539324</v>
       </c>
       <c r="N5" s="21"/>
@@ -19739,23 +19724,23 @@
         <v>73</v>
       </c>
       <c r="I6" s="20">
-        <f>B6/$B6</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J6" s="20">
-        <f>C6/$B6</f>
+        <f t="shared" si="1"/>
         <v>1.0377295492487479</v>
       </c>
       <c r="K6" s="20">
-        <f>D6/$B6</f>
+        <f t="shared" si="2"/>
         <v>4.9288814691151916</v>
       </c>
       <c r="L6" s="20">
-        <f>E6/$B6</f>
+        <f t="shared" si="3"/>
         <v>6.1445742904841403</v>
       </c>
-      <c r="M6" s="73">
-        <f t="shared" si="0"/>
+      <c r="M6" s="69">
+        <f t="shared" si="4"/>
         <v>1.2466467958271239</v>
       </c>
       <c r="N6" s="21"/>
@@ -19801,23 +19786,23 @@
         <v>74</v>
       </c>
       <c r="I7" s="20">
-        <f>B7/$B7</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J7" s="20">
-        <f>C7/$B7</f>
+        <f t="shared" si="1"/>
         <v>1.0470823941898322</v>
       </c>
       <c r="K7" s="20">
-        <f>D7/$B7</f>
+        <f t="shared" si="2"/>
         <v>4.1277235161532682</v>
       </c>
       <c r="L7" s="20">
-        <f>E7/$B7</f>
+        <f t="shared" si="3"/>
         <v>4.8690207863761579</v>
       </c>
-      <c r="M7" s="73">
-        <f t="shared" si="0"/>
+      <c r="M7" s="69">
+        <f t="shared" si="4"/>
         <v>1.1795898556000484</v>
       </c>
       <c r="N7" s="21"/>
@@ -19863,23 +19848,23 @@
         <v>75</v>
       </c>
       <c r="I8" s="20">
-        <f>B8/$B8</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J8" s="20">
-        <f>C8/$B8</f>
+        <f t="shared" si="1"/>
         <v>1.0883816213052384</v>
       </c>
       <c r="K8" s="20">
-        <f>D8/$B8</f>
+        <f t="shared" si="2"/>
         <v>1.2250512145156569</v>
       </c>
       <c r="L8" s="20">
-        <f>E8/$B8</f>
+        <f t="shared" si="3"/>
         <v>1.2780216564237636</v>
       </c>
-      <c r="M8" s="73">
-        <f t="shared" si="0"/>
+      <c r="M8" s="69">
+        <f t="shared" si="4"/>
         <v>1.043239369326326</v>
       </c>
       <c r="N8" s="21"/>
@@ -19925,23 +19910,23 @@
         <v>76</v>
       </c>
       <c r="I9" s="20">
-        <f>B9/$B9</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J9" s="20">
-        <f>C9/$B9</f>
+        <f t="shared" si="1"/>
         <v>0.95233142659039693</v>
       </c>
       <c r="K9" s="20">
-        <f>D9/$B9</f>
+        <f t="shared" si="2"/>
         <v>0.95510487086150109</v>
       </c>
       <c r="L9" s="20">
-        <f>E9/$B9</f>
+        <f t="shared" si="3"/>
         <v>1.0570289478245796</v>
       </c>
-      <c r="M9" s="73">
-        <f t="shared" si="0"/>
+      <c r="M9" s="69">
+        <f t="shared" si="4"/>
         <v>1.1067150635208711</v>
       </c>
       <c r="N9" s="21"/>
@@ -19987,23 +19972,23 @@
         <v>77</v>
       </c>
       <c r="I10" s="20">
-        <f>B10/$B10</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J10" s="20">
-        <f>C10/$B10</f>
+        <f t="shared" si="1"/>
         <v>1.3793103448275863</v>
       </c>
       <c r="K10" s="20">
-        <f>D10/$B10</f>
+        <f t="shared" si="2"/>
         <v>12.206896551724139</v>
       </c>
       <c r="L10" s="20">
-        <f>E10/$B10</f>
+        <f t="shared" si="3"/>
         <v>18.413793103448278</v>
       </c>
-      <c r="M10" s="73">
-        <f t="shared" si="0"/>
+      <c r="M10" s="69">
+        <f t="shared" si="4"/>
         <v>1.5084745762711864</v>
       </c>
       <c r="N10" s="21"/>
@@ -20049,23 +20034,23 @@
         <v>78</v>
       </c>
       <c r="I11" s="20">
-        <f>B11/$B11</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J11" s="20">
-        <f>C11/$B11</f>
+        <f t="shared" si="1"/>
         <v>1.0706467661691543</v>
       </c>
       <c r="K11" s="20">
-        <f>D11/$B11</f>
+        <f t="shared" si="2"/>
         <v>3.9293532338308457</v>
       </c>
       <c r="L11" s="20">
-        <f>E11/$B11</f>
+        <f t="shared" si="3"/>
         <v>5.5562189054726367</v>
       </c>
-      <c r="M11" s="73">
-        <f t="shared" si="0"/>
+      <c r="M11" s="69">
+        <f t="shared" si="4"/>
         <v>1.4140288680678652</v>
       </c>
       <c r="N11" s="21"/>
@@ -20090,7 +20075,7 @@
       <c r="X11" s="8"/>
     </row>
     <row r="12" spans="1:24" ht="18" x14ac:dyDescent="0.2">
-      <c r="A12" s="74" t="s">
+      <c r="A12" s="12" t="s">
         <v>154</v>
       </c>
       <c r="B12" s="3">
@@ -20107,27 +20092,27 @@
       </c>
       <c r="F12" s="20"/>
       <c r="G12" s="21"/>
-      <c r="H12" s="74" t="s">
+      <c r="H12" s="12" t="s">
         <v>154</v>
       </c>
       <c r="I12" s="20">
-        <f>B12/$B12</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J12" s="20">
-        <f>C12/$B12</f>
+        <f t="shared" si="1"/>
         <v>1.2215416028586012</v>
       </c>
       <c r="K12" s="20">
-        <f>D12/$B12</f>
+        <f t="shared" si="2"/>
         <v>10.118938233792752</v>
       </c>
       <c r="L12" s="20">
-        <f>E12/$B12</f>
+        <f t="shared" si="3"/>
         <v>14.344053088310362</v>
       </c>
-      <c r="M12" s="73">
-        <f t="shared" si="0"/>
+      <c r="M12" s="69">
+        <f t="shared" si="4"/>
         <v>1.417545275689855</v>
       </c>
       <c r="N12" s="21"/>
@@ -20173,23 +20158,23 @@
         <v>79</v>
       </c>
       <c r="I13" s="20">
-        <f>B13/$B13</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J13" s="20">
-        <f>C13/$B13</f>
+        <f t="shared" si="1"/>
         <v>1.1012931034482758</v>
       </c>
       <c r="K13" s="20">
-        <f>D13/$B13</f>
+        <f t="shared" si="2"/>
         <v>4.3232758620689653</v>
       </c>
       <c r="L13" s="20">
-        <f>E13/$B13</f>
+        <f t="shared" si="3"/>
         <v>5.0107758620689653</v>
       </c>
-      <c r="M13" s="73">
-        <f t="shared" si="0"/>
+      <c r="M13" s="69">
+        <f t="shared" si="4"/>
         <v>1.1590229312063809</v>
       </c>
       <c r="N13" s="21"/>
@@ -20235,23 +20220,23 @@
         <v>80</v>
       </c>
       <c r="I14" s="20">
-        <f>B14/$B14</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J14" s="20">
-        <f>C14/$B14</f>
+        <f t="shared" si="1"/>
         <v>1.4615384615384615</v>
       </c>
       <c r="K14" s="20">
-        <f>D14/$B14</f>
+        <f t="shared" si="2"/>
         <v>6.0384615384615383</v>
       </c>
       <c r="L14" s="20">
-        <f>E14/$B14</f>
+        <f t="shared" si="3"/>
         <v>7.8461538461538458</v>
       </c>
-      <c r="M14" s="73">
-        <f t="shared" si="0"/>
+      <c r="M14" s="69">
+        <f t="shared" si="4"/>
         <v>1.2993630573248407</v>
       </c>
       <c r="N14" s="21"/>
@@ -20295,8 +20280,8 @@
         <f>GEOMEAN(L2:L14)</f>
         <v>5.5819772016716263</v>
       </c>
-      <c r="M15" s="73">
-        <f t="shared" si="0"/>
+      <c r="M15" s="69">
+        <f t="shared" si="4"/>
         <v>1.3219600193433372</v>
       </c>
       <c r="S15" s="2" t="s">
@@ -20317,199 +20302,199 @@
       <c r="X15" s="8"/>
     </row>
     <row r="18" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G18" s="76"/>
-      <c r="H18" s="76"/>
-      <c r="I18" s="76"/>
-      <c r="J18" s="76"/>
-      <c r="K18" s="76"/>
-      <c r="L18" s="76"/>
-      <c r="M18" s="76"/>
-      <c r="N18" s="76"/>
-      <c r="O18" s="76"/>
-      <c r="P18" s="76"/>
-      <c r="Q18" s="76"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
     </row>
     <row r="19" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G19" s="77"/>
-      <c r="H19" s="77"/>
-      <c r="I19" s="77"/>
-      <c r="J19" s="77"/>
-      <c r="K19" s="77"/>
-      <c r="L19" s="77"/>
-      <c r="M19" s="77"/>
-      <c r="N19" s="77"/>
-      <c r="O19" s="77"/>
-      <c r="P19" s="77"/>
-      <c r="Q19" s="77"/>
+      <c r="G19" s="71"/>
+      <c r="H19" s="71"/>
+      <c r="I19" s="71"/>
+      <c r="J19" s="71"/>
+      <c r="K19" s="71"/>
+      <c r="L19" s="71"/>
+      <c r="M19" s="71"/>
+      <c r="N19" s="71"/>
+      <c r="O19" s="71"/>
+      <c r="P19" s="71"/>
+      <c r="Q19" s="71"/>
     </row>
     <row r="20" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G20" s="77"/>
-      <c r="H20" s="77"/>
-      <c r="I20" s="77"/>
-      <c r="J20" s="77"/>
-      <c r="K20" s="77"/>
-      <c r="L20" s="77"/>
-      <c r="M20" s="77"/>
-      <c r="N20" s="77"/>
-      <c r="O20" s="77"/>
-      <c r="P20" s="77"/>
-      <c r="Q20" s="77"/>
+      <c r="G20" s="71"/>
+      <c r="H20" s="71"/>
+      <c r="I20" s="71"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="71"/>
+      <c r="L20" s="71"/>
+      <c r="M20" s="71"/>
+      <c r="N20" s="71"/>
+      <c r="O20" s="71"/>
+      <c r="P20" s="71"/>
+      <c r="Q20" s="71"/>
     </row>
     <row r="21" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G21" s="77"/>
-      <c r="H21" s="77"/>
-      <c r="I21" s="77"/>
-      <c r="J21" s="77"/>
-      <c r="K21" s="77"/>
-      <c r="L21" s="77"/>
-      <c r="M21" s="77"/>
-      <c r="N21" s="77"/>
-      <c r="O21" s="77"/>
-      <c r="P21" s="77"/>
-      <c r="Q21" s="77"/>
+      <c r="G21" s="71"/>
+      <c r="H21" s="71"/>
+      <c r="I21" s="71"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="71"/>
+      <c r="L21" s="71"/>
+      <c r="M21" s="71"/>
+      <c r="N21" s="71"/>
+      <c r="O21" s="71"/>
+      <c r="P21" s="71"/>
+      <c r="Q21" s="71"/>
     </row>
     <row r="22" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G22" s="77"/>
-      <c r="H22" s="77"/>
-      <c r="I22" s="77"/>
-      <c r="J22" s="77"/>
-      <c r="K22" s="77"/>
-      <c r="L22" s="77"/>
-      <c r="M22" s="77"/>
-      <c r="N22" s="77"/>
-      <c r="O22" s="77"/>
-      <c r="P22" s="77"/>
-      <c r="Q22" s="77"/>
+      <c r="G22" s="71"/>
+      <c r="H22" s="71"/>
+      <c r="I22" s="71"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="71"/>
+      <c r="L22" s="71"/>
+      <c r="M22" s="71"/>
+      <c r="N22" s="71"/>
+      <c r="O22" s="71"/>
+      <c r="P22" s="71"/>
+      <c r="Q22" s="71"/>
     </row>
     <row r="23" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G23" s="77"/>
-      <c r="H23" s="77"/>
-      <c r="I23" s="77"/>
-      <c r="J23" s="77"/>
-      <c r="K23" s="77"/>
-      <c r="L23" s="77"/>
-      <c r="M23" s="77"/>
-      <c r="N23" s="77"/>
-      <c r="O23" s="77"/>
-      <c r="P23" s="77"/>
-      <c r="Q23" s="77"/>
+      <c r="G23" s="71"/>
+      <c r="H23" s="71"/>
+      <c r="I23" s="71"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="71"/>
+      <c r="L23" s="71"/>
+      <c r="M23" s="71"/>
+      <c r="N23" s="71"/>
+      <c r="O23" s="71"/>
+      <c r="P23" s="71"/>
+      <c r="Q23" s="71"/>
     </row>
     <row r="24" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G24" s="77"/>
-      <c r="H24" s="77"/>
-      <c r="I24" s="77"/>
-      <c r="J24" s="77"/>
-      <c r="K24" s="77"/>
-      <c r="L24" s="77"/>
-      <c r="M24" s="77"/>
-      <c r="N24" s="77"/>
-      <c r="O24" s="77"/>
-      <c r="P24" s="77"/>
-      <c r="Q24" s="77"/>
+      <c r="G24" s="71"/>
+      <c r="H24" s="71"/>
+      <c r="I24" s="71"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="71"/>
+      <c r="L24" s="71"/>
+      <c r="M24" s="71"/>
+      <c r="N24" s="71"/>
+      <c r="O24" s="71"/>
+      <c r="P24" s="71"/>
+      <c r="Q24" s="71"/>
     </row>
     <row r="25" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G25" s="77"/>
-      <c r="H25" s="77"/>
-      <c r="I25" s="77"/>
-      <c r="J25" s="77"/>
-      <c r="K25" s="77"/>
-      <c r="L25" s="77"/>
-      <c r="M25" s="77"/>
-      <c r="N25" s="77"/>
-      <c r="O25" s="77"/>
-      <c r="P25" s="77"/>
-      <c r="Q25" s="77"/>
+      <c r="G25" s="71"/>
+      <c r="H25" s="71"/>
+      <c r="I25" s="71"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="71"/>
+      <c r="L25" s="71"/>
+      <c r="M25" s="71"/>
+      <c r="N25" s="71"/>
+      <c r="O25" s="71"/>
+      <c r="P25" s="71"/>
+      <c r="Q25" s="71"/>
     </row>
     <row r="26" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G26" s="77"/>
-      <c r="H26" s="77"/>
-      <c r="I26" s="77"/>
-      <c r="J26" s="77"/>
-      <c r="K26" s="77"/>
-      <c r="L26" s="77"/>
-      <c r="M26" s="77"/>
-      <c r="N26" s="77"/>
-      <c r="O26" s="77"/>
-      <c r="P26" s="77"/>
-      <c r="Q26" s="77"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="71"/>
+      <c r="L26" s="71"/>
+      <c r="M26" s="71"/>
+      <c r="N26" s="71"/>
+      <c r="O26" s="71"/>
+      <c r="P26" s="71"/>
+      <c r="Q26" s="71"/>
     </row>
     <row r="27" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G27" s="77"/>
-      <c r="H27" s="77"/>
-      <c r="I27" s="77"/>
-      <c r="J27" s="77"/>
-      <c r="K27" s="77"/>
-      <c r="L27" s="77"/>
-      <c r="M27" s="77"/>
-      <c r="N27" s="77"/>
-      <c r="O27" s="77"/>
-      <c r="P27" s="77"/>
-      <c r="Q27" s="77"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="71"/>
+      <c r="L27" s="71"/>
+      <c r="M27" s="71"/>
+      <c r="N27" s="71"/>
+      <c r="O27" s="71"/>
+      <c r="P27" s="71"/>
+      <c r="Q27" s="71"/>
     </row>
     <row r="28" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G28" s="77"/>
-      <c r="H28" s="77"/>
-      <c r="I28" s="77"/>
-      <c r="J28" s="77"/>
-      <c r="K28" s="77"/>
-      <c r="L28" s="77"/>
-      <c r="M28" s="77"/>
-      <c r="N28" s="77"/>
-      <c r="O28" s="77"/>
-      <c r="P28" s="77"/>
-      <c r="Q28" s="77"/>
+      <c r="G28" s="71"/>
+      <c r="H28" s="71"/>
+      <c r="I28" s="71"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="71"/>
+      <c r="L28" s="71"/>
+      <c r="M28" s="71"/>
+      <c r="N28" s="71"/>
+      <c r="O28" s="71"/>
+      <c r="P28" s="71"/>
+      <c r="Q28" s="71"/>
     </row>
     <row r="29" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G29" s="77"/>
-      <c r="H29" s="77"/>
-      <c r="I29" s="77"/>
-      <c r="J29" s="77"/>
-      <c r="K29" s="77"/>
-      <c r="L29" s="77"/>
-      <c r="M29" s="77"/>
-      <c r="N29" s="77"/>
-      <c r="O29" s="77"/>
-      <c r="P29" s="77"/>
-      <c r="Q29" s="77"/>
+      <c r="G29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="71"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="71"/>
+      <c r="L29" s="71"/>
+      <c r="M29" s="71"/>
+      <c r="N29" s="71"/>
+      <c r="O29" s="71"/>
+      <c r="P29" s="71"/>
+      <c r="Q29" s="71"/>
     </row>
     <row r="30" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G30" s="77"/>
-      <c r="H30" s="77"/>
-      <c r="I30" s="77"/>
-      <c r="J30" s="77"/>
-      <c r="K30" s="77"/>
-      <c r="L30" s="77"/>
-      <c r="M30" s="77"/>
-      <c r="N30" s="77"/>
-      <c r="O30" s="77"/>
-      <c r="P30" s="77"/>
-      <c r="Q30" s="77"/>
+      <c r="G30" s="71"/>
+      <c r="H30" s="71"/>
+      <c r="I30" s="71"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="71"/>
+      <c r="L30" s="71"/>
+      <c r="M30" s="71"/>
+      <c r="N30" s="71"/>
+      <c r="O30" s="71"/>
+      <c r="P30" s="71"/>
+      <c r="Q30" s="71"/>
     </row>
     <row r="31" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G31" s="77"/>
-      <c r="H31" s="77"/>
-      <c r="I31" s="77"/>
-      <c r="J31" s="77"/>
-      <c r="K31" s="77"/>
-      <c r="L31" s="77"/>
-      <c r="M31" s="77"/>
-      <c r="N31" s="77"/>
-      <c r="O31" s="77"/>
-      <c r="P31" s="77"/>
-      <c r="Q31" s="77"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="71"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="71"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="71"/>
+      <c r="M31" s="71"/>
+      <c r="N31" s="71"/>
+      <c r="O31" s="71"/>
+      <c r="P31" s="71"/>
+      <c r="Q31" s="71"/>
     </row>
     <row r="32" spans="7:17" ht="18" x14ac:dyDescent="0.2">
-      <c r="G32" s="77"/>
-      <c r="H32" s="77"/>
-      <c r="I32" s="77"/>
-      <c r="J32" s="77"/>
-      <c r="K32" s="77"/>
-      <c r="L32" s="77"/>
-      <c r="M32" s="77"/>
-      <c r="N32" s="77"/>
-      <c r="O32" s="77"/>
-      <c r="P32" s="77"/>
-      <c r="Q32" s="77"/>
+      <c r="G32" s="71"/>
+      <c r="H32" s="71"/>
+      <c r="I32" s="71"/>
+      <c r="J32" s="71"/>
+      <c r="K32" s="71"/>
+      <c r="L32" s="71"/>
+      <c r="M32" s="71"/>
+      <c r="N32" s="71"/>
+      <c r="O32" s="71"/>
+      <c r="P32" s="71"/>
+      <c r="Q32" s="71"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20544,17 +20529,17 @@
     </row>
     <row r="2" spans="2:17" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="8"/>
-      <c r="C2" s="70" t="s">
+      <c r="C2" s="74" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="68" t="s">
+      <c r="D2" s="72" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="69"/>
+      <c r="E2" s="73"/>
     </row>
     <row r="3" spans="2:17" ht="18" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="70"/>
+      <c r="C3" s="74"/>
       <c r="D3" s="6" t="s">
         <v>83</v>
       </c>

</xml_diff>